<commit_message>
fix typo in author name
</commit_message>
<xml_diff>
--- a/data/source_papers.xlsx
+++ b/data/source_papers.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maa77\Documents\.MIJN BESTANDEN\Wiskunde &amp; Informatica\NAS website\GitHub repo\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A38629C-4F7A-4032-9DCD-FC4B2B9FC914}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{468F3714-55F1-4486-9090-6E8A29EE3219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5391,9 +5391,6 @@
     <t>10.1109/tnsm.2025.3607004</t>
   </si>
   <si>
-    <t>X. Liu, R. Kooij, P.V. Mieghem</t>
-  </si>
-  <si>
     <t>Node-Reliability: Monte Carlo, Laplace, and Stochastic Approximations and a Greedy Link-Augmentation Strategy</t>
   </si>
   <si>
@@ -5464,6 +5461,9 @@
   </si>
   <si>
     <t>B.L. Chang, L. Yang, M. Sensi, M.A. Achterberg, F. Wang, M. Rinaldi, P. Van Mieghem</t>
+  </si>
+  <si>
+    <t>X. Liu, R. Kooij, P. Van Mieghem</t>
   </si>
 </sst>
 </file>
@@ -5869,16 +5869,16 @@
     </row>
     <row r="2" spans="1:12" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>1802</v>
+        <v>1801</v>
       </c>
       <c r="B2" t="s">
-        <v>1809</v>
+        <v>1808</v>
       </c>
       <c r="C2">
         <v>2026</v>
       </c>
       <c r="D2" t="s">
-        <v>1810</v>
+        <v>1809</v>
       </c>
       <c r="F2" t="s">
         <v>750</v>
@@ -5889,19 +5889,19 @@
     </row>
     <row r="3" spans="1:12" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>1801</v>
+        <v>1800</v>
       </c>
       <c r="B3" t="s">
-        <v>1800</v>
+        <v>1799</v>
       </c>
       <c r="C3">
         <v>2026</v>
       </c>
       <c r="D3" t="s">
-        <v>1799</v>
+        <v>1798</v>
       </c>
       <c r="E3" t="s">
-        <v>1798</v>
+        <v>1797</v>
       </c>
       <c r="F3" t="s">
         <v>2</v>
@@ -5913,7 +5913,7 @@
         <v>2</v>
       </c>
       <c r="I3" t="s">
-        <v>1797</v>
+        <v>1796</v>
       </c>
       <c r="J3" t="s">
         <v>1003</v>
@@ -5924,10 +5924,10 @@
     </row>
     <row r="4" spans="1:12" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>1796</v>
+        <v>1795</v>
       </c>
       <c r="B4" t="s">
-        <v>1795</v>
+        <v>1794</v>
       </c>
       <c r="C4">
         <v>2025</v>
@@ -5936,7 +5936,7 @@
         <v>854</v>
       </c>
       <c r="E4" t="s">
-        <v>1794</v>
+        <v>1793</v>
       </c>
       <c r="F4" t="s">
         <v>2</v>
@@ -5948,7 +5948,7 @@
         <v>10</v>
       </c>
       <c r="I4" t="s">
-        <v>1793</v>
+        <v>1792</v>
       </c>
       <c r="J4" t="s">
         <v>806</v>
@@ -5959,10 +5959,10 @@
     </row>
     <row r="5" spans="1:12" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>1792</v>
+        <v>1791</v>
       </c>
       <c r="B5" t="s">
-        <v>1791</v>
+        <v>1790</v>
       </c>
       <c r="C5">
         <v>2025</v>
@@ -5971,7 +5971,7 @@
         <v>59</v>
       </c>
       <c r="E5" t="s">
-        <v>1790</v>
+        <v>1789</v>
       </c>
       <c r="F5" t="s">
         <v>2</v>
@@ -5983,7 +5983,7 @@
         <v>9</v>
       </c>
       <c r="I5" t="s">
-        <v>1789</v>
+        <v>1788</v>
       </c>
       <c r="J5" t="s">
         <v>903</v>
@@ -5994,10 +5994,10 @@
     </row>
     <row r="6" spans="1:12" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>1788</v>
+        <v>1787</v>
       </c>
       <c r="B6" t="s">
-        <v>1787</v>
+        <v>1811</v>
       </c>
       <c r="C6">
         <v>2026</v>
@@ -6416,10 +6416,10 @@
     </row>
     <row r="19" spans="1:12" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
+        <v>1804</v>
+      </c>
+      <c r="B19" t="s">
         <v>1805</v>
-      </c>
-      <c r="B19" t="s">
-        <v>1806</v>
       </c>
       <c r="C19">
         <v>2024</v>
@@ -6428,7 +6428,7 @@
         <v>13</v>
       </c>
       <c r="E19" t="s">
-        <v>1807</v>
+        <v>1806</v>
       </c>
       <c r="F19" t="s">
         <v>2</v>
@@ -6486,7 +6486,7 @@
         <v>2024</v>
       </c>
       <c r="D21" t="s">
-        <v>1804</v>
+        <v>1803</v>
       </c>
       <c r="F21" t="s">
         <v>750</v>
@@ -6494,7 +6494,7 @@
     </row>
     <row r="22" spans="1:12" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>1808</v>
+        <v>1807</v>
       </c>
       <c r="B22" t="s">
         <v>1750</v>
@@ -6503,7 +6503,7 @@
         <v>2024</v>
       </c>
       <c r="D22" t="s">
-        <v>1803</v>
+        <v>1802</v>
       </c>
       <c r="F22" t="s">
         <v>750</v>
@@ -7987,7 +7987,7 @@
         <v>826</v>
       </c>
       <c r="B68" t="s">
-        <v>1811</v>
+        <v>1810</v>
       </c>
       <c r="C68">
         <v>2022</v>

</xml_diff>